<commit_message>
fix: reformat Kyrgyz names to correct Имя ИмяОтца уулу/кызы order
</commit_message>
<xml_diff>
--- a/ЦНСВ БД.xlsx
+++ b/ЦНСВ БД.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абдилова Свветлана </t>
+          <t>Абдилова Светлана</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Анаркадый уулу Адилет </t>
+          <t>Адилет Анаркадый уулу</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Шергазы уулу Тилктеш </t>
+          <t>Тилктеш Шергазы уулу</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жодатбек уулу Нур </t>
+          <t>Нур Жодатбек уулу</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Женишбек уулу Азамат </t>
+          <t>Азамат Женишбек уулу</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абдыгапыр кызы Фарида </t>
+          <t>Фарида Абдыгапыр кызы</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Арапбай кызы Аида </t>
+          <t>Аида Арапбай кызы</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Азим кызы Нуржамал </t>
+          <t>Нуржамал Азим кызы</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бактыбек кызы Бурулай </t>
+          <t>Бурулай Бактыбек кызы</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кубанычбек кызы Элиза </t>
+          <t>Элиза Кубанычбек кызы</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мурзакарим кызы Нуржан </t>
+          <t>Нуржан Мурзакарим кызы</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абдумалик уулу Абдуллажан </t>
+          <t>Абдуллажан Абдумалик уулу</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кабыл уулу Айтмамат </t>
+          <t>Айтмамат Кабыл уулу</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Реджапай уулу Абубакир </t>
+          <t>Абубакир Реджапай уулу</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="C71" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Базарбек уулу Азамат </t>
+          <t>Азамат Базарбек уулу</t>
         </is>
       </c>
       <c r="D71" s="13" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C87" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жайлообек уулу Болотбек </t>
+          <t>Болотбек Жайлообек уулу</t>
         </is>
       </c>
       <c r="D87" s="15" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="C88" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жангарач уулу Исабек </t>
+          <t>Исабек Жангарач уулу</t>
         </is>
       </c>
       <c r="D88" s="15" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="C96" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эркинбек уулу Кубатбек </t>
+          <t>Кубатбек Эркинбек уулу</t>
         </is>
       </c>
       <c r="D96" s="15" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абдыбек кызы Адина </t>
+          <t>Адина Абдыбек кызы</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бектурсун кызы Жазгул </t>
+          <t>Жазгул Бектурсун кызы</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Журсунбек кызы Динара </t>
+          <t>Динара Журсунбек кызы</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абылжан кызы Айгул </t>
+          <t>Айгул Абылжан кызы</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жумадил кызы Чынаркул </t>
+          <t>Чынаркул Жумадил кызы</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сапарбек уулу Эрназар </t>
+          <t>Эрназар Сапарбек уулу</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нуридин кызы Айдай </t>
+          <t>Айдай Нуридин кызы</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Камбаралы уулу Манасбек </t>
+          <t>Манасбек Камбаралы уулу</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ишенбай уулу Жыргалбек </t>
+          <t>Жыргалбек Ишенбай уулу</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рыскелди уулу Мирлан </t>
+          <t>Мирлан Рыскелди уулу</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
@@ -7127,7 +7127,7 @@
       </c>
       <c r="C206" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кубанычбек уулу Тынарбек </t>
+          <t>Тынарбек Кубанычбек уулу</t>
         </is>
       </c>
       <c r="D206" s="13" t="inlineStr">
@@ -7255,7 +7255,7 @@
       </c>
       <c r="C210" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жумак уулу Максат </t>
+          <t>Максат Жумак уулу</t>
         </is>
       </c>
       <c r="D210" s="13" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кадирберди кызы Махиро </t>
+          <t>Махиро Кадирберди кызы</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Элинжан кызы Айчурок </t>
+          <t>Айчурок Элинжан кызы</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эржин кызы Асылкан </t>
+          <t>Асылкан Эржин кызы</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
@@ -7863,7 +7863,7 @@
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Дажап кызы Азиза </t>
+          <t>Азиза Дажап кызы</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Саламбек кыз Мираида </t>
+          <t>Мираида Саламбек кызы</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абдимажит кызы Жумагул </t>
+          <t>Жумагул Абдимажит кызы</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Акылбек кызы Айгерим </t>
+          <t>Айгерим Акылбек кызы</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маматшукур кызы Канышай </t>
+          <t>Канышай Маматшукур кызы</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
@@ -9975,7 +9975,7 @@
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Асыбек кызы Жибек </t>
+          <t>Жибек Асыбек кызы</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ноокенбай уулу Нурсултан </t>
+          <t>Нурсултан Ноокенбай уулу</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мадылбек уулу Адилет </t>
+          <t>Адилет Мадылбек уулу</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Билимбек уулу Мухаммадабдурах</t>
+          <t>Мухаммадабдурах Билимбек уулу</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
@@ -11159,7 +11159,7 @@
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Абдыкадыр уулу Азамат </t>
+          <t>Азамат Абдыкадыр уулу</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
@@ -11447,7 +11447,7 @@
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Палывжан уулу Анваржан </t>
+          <t>Анваржан Палывжан уулу</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бактыбек уулу Мирбек </t>
+          <t>Мирбек Бактыбек уулу</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
@@ -11575,7 +11575,7 @@
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Курманбек уулу Суусарбек </t>
+          <t>Суусарбек Курманбек уулу</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
@@ -12023,7 +12023,7 @@
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Камал уулу Улукман </t>
+          <t>Улукман Камал уулу</t>
         </is>
       </c>
       <c r="D359" s="4" t="inlineStr">
@@ -12247,7 +12247,7 @@
       </c>
       <c r="C366" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Садырбек кызы Омуркан </t>
+          <t>Омуркан Садырбек кызы</t>
         </is>
       </c>
       <c r="D366" s="4" t="inlineStr">
@@ -12343,7 +12343,7 @@
       </c>
       <c r="C369" s="4" t="inlineStr">
         <is>
-          <t>Алтынбек кызы Айдана</t>
+          <t>Айдана Алтынбек кызы</t>
         </is>
       </c>
       <c r="D369" s="4" t="inlineStr">
@@ -12503,7 +12503,7 @@
       </c>
       <c r="C374" s="4" t="inlineStr">
         <is>
-          <t>Муталипжан кызы Мухлис</t>
+          <t>Мухлис Муталипжан кызы</t>
         </is>
       </c>
       <c r="D374" s="4" t="inlineStr">
@@ -12631,7 +12631,7 @@
       </c>
       <c r="C378" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жанторо уулу Тенирберди </t>
+          <t>Тенирберди Жанторо уулу</t>
         </is>
       </c>
       <c r="D378" s="4" t="inlineStr">
@@ -12695,7 +12695,7 @@
       </c>
       <c r="C380" s="4" t="inlineStr">
         <is>
-          <t>Дайырбек уулу Чингизхан</t>
+          <t>Чингизхан Дайырбек уулу</t>
         </is>
       </c>
       <c r="D380" s="4" t="inlineStr">
@@ -13495,7 +13495,7 @@
       </c>
       <c r="C405" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Асек уулу Омурзак </t>
+          <t>Омурзак Асек уулу</t>
         </is>
       </c>
       <c r="D405" s="4" t="inlineStr">
@@ -13527,7 +13527,7 @@
       </c>
       <c r="C406" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жумабек уулу Торобек </t>
+          <t>Торобек Жумабек уулу</t>
         </is>
       </c>
       <c r="D406" s="4" t="inlineStr">
@@ -14455,7 +14455,7 @@
       </c>
       <c r="C435" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бактыбек уулу Айтолду </t>
+          <t>Айтолду Бактыбек уулу</t>
         </is>
       </c>
       <c r="D435" s="5" t="inlineStr">
@@ -14743,7 +14743,7 @@
       </c>
       <c r="C444" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нурбек уулу Зайырбек </t>
+          <t>Зайырбек Нурбек уулу</t>
         </is>
       </c>
       <c r="D444" s="13" t="inlineStr">
@@ -14775,7 +14775,7 @@
       </c>
       <c r="C445" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Турдалы уулу Арстанбек </t>
+          <t>Арстанбек Турдалы уулу</t>
         </is>
       </c>
       <c r="D445" s="13" t="inlineStr">
@@ -14807,7 +14807,7 @@
       </c>
       <c r="C446" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чынгыз уулу Кочкунбек </t>
+          <t>Кочкунбек Чынгыз уулу</t>
         </is>
       </c>
       <c r="D446" s="13" t="inlineStr">
@@ -15351,7 +15351,7 @@
       </c>
       <c r="C463" s="13" t="inlineStr">
         <is>
-          <t>Жаныбек уулу Эржан</t>
+          <t>Эржан Жаныбек уулу</t>
         </is>
       </c>
       <c r="D463" s="13" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="C477" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эралы кызы Каныкей </t>
+          <t>Каныкей Эралы кызы</t>
         </is>
       </c>
       <c r="D477" s="13" t="inlineStr">
@@ -16183,7 +16183,7 @@
       </c>
       <c r="C489" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нурбек кызы Чолпонай </t>
+          <t>Чолпонай Нурбек кызы</t>
         </is>
       </c>
       <c r="D489" s="13" t="inlineStr">
@@ -16855,7 +16855,7 @@
       </c>
       <c r="C510" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Куванычбек кызы Айперим </t>
+          <t>Айперим Куванычбек кызы</t>
         </is>
       </c>
       <c r="D510" s="13" t="inlineStr">
@@ -17559,7 +17559,7 @@
       </c>
       <c r="C532" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Азамат уулу Сталбек </t>
+          <t>Сталбек Азамат уулу</t>
         </is>
       </c>
       <c r="D532" s="15" t="inlineStr">
@@ -18263,7 +18263,7 @@
       </c>
       <c r="C554" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эркин уулу Аскат </t>
+          <t>Аскат Эркин уулу</t>
         </is>
       </c>
       <c r="D554" s="4" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="C567" s="4" t="inlineStr">
         <is>
-          <t>Акматалы уулу Женишбек</t>
+          <t>Женишбек Акматалы уулу</t>
         </is>
       </c>
       <c r="D567" s="4" t="inlineStr">
@@ -19127,7 +19127,7 @@
       </c>
       <c r="C581" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Джайлообек уулу Эрлан </t>
+          <t>Эрлан Джайлообек уулу</t>
         </is>
       </c>
       <c r="D581" s="4" t="inlineStr">
@@ -19251,7 +19251,7 @@
       </c>
       <c r="C585" s="4" t="inlineStr">
         <is>
-          <t>Акылбек уулу Бекбоо</t>
+          <t>Бекбоо Акылбек уулу</t>
         </is>
       </c>
       <c r="D585" s="4" t="inlineStr">
@@ -19315,7 +19315,7 @@
       </c>
       <c r="C587" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маратбек уулу Бексултан </t>
+          <t>Бексултан Маратбек уулу</t>
         </is>
       </c>
       <c r="D587" s="4" t="inlineStr">
@@ -19827,7 +19827,7 @@
       </c>
       <c r="C603" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сагынбек кызы Акылай </t>
+          <t>Акылай Сагынбек кызы</t>
         </is>
       </c>
       <c r="D603" s="4" t="inlineStr">
@@ -20115,7 +20115,7 @@
       </c>
       <c r="C612" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Самудин уулу Азис </t>
+          <t>Азис Самудин уулу</t>
         </is>
       </c>
       <c r="D612" s="4" t="inlineStr">
@@ -20211,7 +20211,7 @@
       </c>
       <c r="C615" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сагынбек уулу Азим </t>
+          <t>Азим Сагынбек уулу</t>
         </is>
       </c>
       <c r="D615" s="4" t="inlineStr">
@@ -20595,7 +20595,7 @@
       </c>
       <c r="C627" s="4" t="inlineStr">
         <is>
-          <t>Турусбек кызы Нурзада</t>
+          <t>Нурзада Турусбек кызы</t>
         </is>
       </c>
       <c r="D627" s="4" t="inlineStr">
@@ -20755,7 +20755,7 @@
       </c>
       <c r="C632" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сиезбек уулу Эрнас </t>
+          <t>Эрнас Сиезбек уулу</t>
         </is>
       </c>
       <c r="D632" s="4" t="inlineStr">
@@ -20979,7 +20979,7 @@
       </c>
       <c r="C639" s="4" t="inlineStr">
         <is>
-          <t>Камчыбек кызы Айзаада</t>
+          <t>Айзаада Камчыбек кызы</t>
         </is>
       </c>
       <c r="D639" s="4" t="inlineStr">
@@ -21043,7 +21043,7 @@
       </c>
       <c r="C641" s="4" t="inlineStr">
         <is>
-          <t>Жыргалбек уулу Эрнис</t>
+          <t>Эрнис Жыргалбек уулу</t>
         </is>
       </c>
       <c r="D641" s="4" t="inlineStr">
@@ -21299,7 +21299,7 @@
       </c>
       <c r="C649" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Токтогул кызы Адинай </t>
+          <t>Адинай Токтогул кызы</t>
         </is>
       </c>
       <c r="D649" s="4" t="inlineStr">
@@ -21491,7 +21491,7 @@
       </c>
       <c r="C655" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ишен уулу Эдилбек </t>
+          <t>Эдилбек Ишен уулу</t>
         </is>
       </c>
       <c r="D655" s="4" t="inlineStr">
@@ -21651,7 +21651,7 @@
       </c>
       <c r="C660" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Батырбек уулу Элеман </t>
+          <t>Элеман Батырбек уулу</t>
         </is>
       </c>
       <c r="D660" s="4" t="inlineStr">
@@ -21843,7 +21843,7 @@
       </c>
       <c r="C666" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тагайбек уулу Бообек </t>
+          <t>Бообек Тагайбек уулу</t>
         </is>
       </c>
       <c r="D666" s="4" t="inlineStr">
@@ -21875,7 +21875,7 @@
       </c>
       <c r="C667" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жумабай уулу Марсбек </t>
+          <t>Марсбек Жумабай уулу</t>
         </is>
       </c>
       <c r="D667" s="4" t="inlineStr">
@@ -21939,7 +21939,7 @@
       </c>
       <c r="C669" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ишеналы уулу Беккалнур </t>
+          <t>Беккалнур Ишеналы уулу</t>
         </is>
       </c>
       <c r="D669" s="4" t="inlineStr">
@@ -21971,7 +21971,7 @@
       </c>
       <c r="C670" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ишеналы уулу Беккалнур </t>
+          <t>Беккалнур Ишеналы уулу</t>
         </is>
       </c>
       <c r="D670" s="4" t="inlineStr">
@@ -22003,7 +22003,7 @@
       </c>
       <c r="C671" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Акыш уулу Актилек </t>
+          <t>Актилек Акыш уулу</t>
         </is>
       </c>
       <c r="D671" s="4" t="inlineStr">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="C677" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бектен уулу Мирбек </t>
+          <t>Мирбек Бектен уулу</t>
         </is>
       </c>
       <c r="D677" s="4" t="inlineStr">
@@ -22487,7 +22487,7 @@
       </c>
       <c r="C686" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Авазбек уулу Азамат </t>
+          <t>Азамат Авазбек уулу</t>
         </is>
       </c>
       <c r="D686" s="4" t="inlineStr">
@@ -23351,7 +23351,7 @@
       </c>
       <c r="C713" s="4" t="inlineStr">
         <is>
-          <t>Шабданбек уулу Эсенжан</t>
+          <t>Эсенжан Шабданбек уулу</t>
         </is>
       </c>
       <c r="D713" s="4" t="inlineStr">
@@ -24023,7 +24023,7 @@
       </c>
       <c r="C734" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жайлообек уулу Бектурган </t>
+          <t>Бектурган Жайлообек уулу</t>
         </is>
       </c>
       <c r="D734" s="4" t="inlineStr">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="C736" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Азамат уулу Арген </t>
+          <t>Арген Азамат уулу</t>
         </is>
       </c>
       <c r="D736" s="4" t="inlineStr">
@@ -24151,7 +24151,7 @@
       </c>
       <c r="C738" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мыйманбай кызы Токтаим </t>
+          <t>Токтаим Мыйманбай кызы</t>
         </is>
       </c>
       <c r="D738" s="4" t="inlineStr">
@@ -24311,7 +24311,7 @@
       </c>
       <c r="C743" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Таашыбек уулу Кутман </t>
+          <t>Кутман Таашыбек уулу</t>
         </is>
       </c>
       <c r="D743" s="4" t="inlineStr">
@@ -24343,7 +24343,7 @@
       </c>
       <c r="C744" s="4" t="inlineStr">
         <is>
-          <t>Жылдызбек уулу Орозбек</t>
+          <t>Орозбек Жылдызбек уулу</t>
         </is>
       </c>
       <c r="D744" s="4" t="inlineStr">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="C748" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Жапар уулу Бектур </t>
+          <t>Бектур Жапар уулу</t>
         </is>
       </c>
       <c r="D748" s="4" t="inlineStr">
@@ -24663,7 +24663,7 @@
       </c>
       <c r="C754" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Турдумамат кызы Абиба </t>
+          <t>Абиба Турдумамат кызы</t>
         </is>
       </c>
       <c r="D754" s="4" t="inlineStr">
@@ -24855,7 +24855,7 @@
       </c>
       <c r="C760" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">тронин Александр Викторович </t>
+          <t>Тронин Александр Викторович</t>
         </is>
       </c>
       <c r="D760" s="4" t="inlineStr">
@@ -24887,7 +24887,7 @@
       </c>
       <c r="C761" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Догдурбай у Калыгул </t>
+          <t>Калыгул Догдурбай уулу</t>
         </is>
       </c>
       <c r="D761" s="4" t="inlineStr">
@@ -25015,7 +25015,7 @@
       </c>
       <c r="C765" s="4" t="inlineStr">
         <is>
-          <t>Сатымкулова Мира  Балтабаевна</t>
+          <t>Сатымкулова Мира Балтабаевна</t>
         </is>
       </c>
       <c r="D765" s="4" t="inlineStr">
@@ -25047,7 +25047,7 @@
       </c>
       <c r="C766" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Туратбек у Омурбек </t>
+          <t>Омурбек Туратбек уулу</t>
         </is>
       </c>
       <c r="D766" s="4" t="inlineStr">
@@ -25079,7 +25079,7 @@
       </c>
       <c r="C767" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Назаралиева  Сабырбү  </t>
+          <t>Назаралиева Сабырбү</t>
         </is>
       </c>
       <c r="D767" s="4" t="inlineStr">
@@ -25111,7 +25111,7 @@
       </c>
       <c r="C768" s="4" t="inlineStr">
         <is>
-          <t>Акылбек уулу Бекмамат</t>
+          <t>Бекмамат Акылбек уулу</t>
         </is>
       </c>
       <c r="D768" s="4" t="inlineStr">
@@ -25943,7 +25943,7 @@
       </c>
       <c r="C794" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тынштык кызы Элзат </t>
+          <t>Элзат Тынштык кызы</t>
         </is>
       </c>
       <c r="D794" s="4" t="inlineStr">
@@ -25975,7 +25975,7 @@
       </c>
       <c r="C795" s="4" t="inlineStr">
         <is>
-          <t>Нурдөөлөт у Өскөнбек</t>
+          <t>Өскөнбек Нурдөөлөт уулу</t>
         </is>
       </c>
       <c r="D795" s="4" t="inlineStr">
@@ -26199,7 +26199,7 @@
       </c>
       <c r="C802" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Авазбек кызы Гулзада </t>
+          <t>Гулзада Авазбек кызы</t>
         </is>
       </c>
       <c r="D802" s="4" t="inlineStr">
@@ -26359,7 +26359,7 @@
       </c>
       <c r="C807" s="4" t="inlineStr">
         <is>
-          <t>Кудайберген кызы Алмагүл</t>
+          <t>Алмагүл Кудайберген кызы</t>
         </is>
       </c>
       <c r="D807" s="4" t="inlineStr">
@@ -26423,7 +26423,7 @@
       </c>
       <c r="C809" s="4" t="inlineStr">
         <is>
-          <t>Сагынбек кызы Эркинай</t>
+          <t>Эркинай Сагынбек кызы</t>
         </is>
       </c>
       <c r="D809" s="4" t="inlineStr">
@@ -26455,7 +26455,7 @@
       </c>
       <c r="C810" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Самыйбек уулу Эсенбек </t>
+          <t>Эсенбек Самыйбек уулу</t>
         </is>
       </c>
       <c r="D810" s="4" t="inlineStr">
@@ -26487,7 +26487,7 @@
       </c>
       <c r="C811" s="4" t="inlineStr">
         <is>
-          <t>Олжобай кызы Бактыгүл</t>
+          <t>Бактыгүл Олжобай кызы</t>
         </is>
       </c>
       <c r="D811" s="4" t="inlineStr">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="C817" s="4" t="inlineStr">
         <is>
-          <t>Курманбек кызы Жазгүл</t>
+          <t>Жазгүл Курманбек кызы</t>
         </is>
       </c>
       <c r="D817" s="4" t="inlineStr">
@@ -26839,7 +26839,7 @@
       </c>
       <c r="C822" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Эрболот уулу Элдос </t>
+          <t>Элдос Эрболот уулу</t>
         </is>
       </c>
       <c r="D822" s="4" t="inlineStr">
@@ -26903,7 +26903,7 @@
       </c>
       <c r="C824" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аскат уулу Алтынбек </t>
+          <t>Алтынбек Аскат уулу</t>
         </is>
       </c>
       <c r="D824" s="4" t="inlineStr">
@@ -26935,7 +26935,7 @@
       </c>
       <c r="C825" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аскат уулу Эмил </t>
+          <t>Эмил Аскат уулу</t>
         </is>
       </c>
       <c r="D825" s="4" t="inlineStr">

</xml_diff>

<commit_message>
fix: correct names for ЦС № 000735 and ЦС № 000293
</commit_message>
<xml_diff>
--- a/ЦНСВ БД.xlsx
+++ b/ЦНСВ БД.xlsx
@@ -11991,7 +11991,7 @@
       </c>
       <c r="C358" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Нурланв Нуржигит </t>
+          <t>Нурланов Нуржигит</t>
         </is>
       </c>
       <c r="D358" s="4" t="inlineStr">
@@ -26135,7 +26135,7 @@
       </c>
       <c r="C800" s="4" t="inlineStr">
         <is>
-          <t>Токтомамбетов Нуржгит Нурдөөлөтович</t>
+          <t>Токтомамбетов Нуржигит Нурдөөлөтович</t>
         </is>
       </c>
       <c r="D800" s="4" t="inlineStr">

</xml_diff>